<commit_message>
Urunler sayfasi b2b ye göre duzenlendi
</commit_message>
<xml_diff>
--- a/public/templates/toptanci-urun-import-sablonu.xlsx
+++ b/public/templates/toptanci-urun-import-sablonu.xlsx
@@ -3,7 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Urunler" sheetId="1" r:id="rId1"/>
+    <sheet name="urunler" sheetId="1" r:id="rId1"/>
+    <sheet name="talimatlar" sheetId="2" r:id="rId2"/>
+    <sheet name="kategori_listesi" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +399,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:V4"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" customWidth="1"/>
+    <col min="4" max="4" width="28.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="40.83203125" customWidth="1"/>
+    <col min="7" max="7" width="40.83203125" customWidth="1"/>
+    <col min="8" max="8" width="40.83203125" customWidth="1"/>
+    <col min="9" max="9" width="30.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="20.83203125" customWidth="1"/>
+    <col min="12" max="12" width="18.83203125" customWidth="1"/>
+    <col min="13" max="13" width="18.83203125" customWidth="1"/>
+    <col min="14" max="14" width="20.83203125" customWidth="1"/>
+    <col min="15" max="15" width="16.83203125" customWidth="1"/>
+    <col min="16" max="16" width="22.83203125" customWidth="1"/>
+    <col min="17" max="17" width="22.83203125" customWidth="1"/>
+    <col min="18" max="18" width="14.83203125" customWidth="1"/>
+    <col min="19" max="19" width="14.83203125" customWidth="1"/>
+    <col min="20" max="20" width="14.83203125" customWidth="1"/>
+    <col min="21" max="21" width="14.83203125" customWidth="1"/>
+    <col min="22" max="22" width="10.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,22 +460,37 @@
         <v>alt_kategori</v>
       </c>
       <c r="L1" t="str">
+        <v>tedarikci</v>
+      </c>
+      <c r="M1" t="str">
         <v>urun_tipi</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>alis_fiyat_seviyesi</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>alis_fiyati</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
+        <v>satis_fiyati_musteri</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>satis_fiyati_alt_bayi</v>
+      </c>
+      <c r="R1" t="str">
         <v>kutu_ici_adet</v>
       </c>
-      <c r="P1" t="str">
+      <c r="S1" t="str">
         <v>koli_ici_kutu</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="T1" t="str">
         <v>palet_ici_koli</v>
+      </c>
+      <c r="U1" t="str">
+        <v>stok_miktari</v>
+      </c>
+      <c r="V1" t="str">
+        <v>aktif</v>
       </c>
     </row>
     <row r="2">
@@ -457,28 +498,28 @@
         <v>CHEESE-001</v>
       </c>
       <c r="B2" t="str">
-        <v>Frambuazli Cheesecake</v>
+        <v>Frambuazlı Cheesecake</v>
       </c>
       <c r="C2" t="str">
-        <v>Himbeer-Kasekuchen</v>
+        <v>Himbeer-Käsekuchen</v>
       </c>
       <c r="D2" t="str">
         <v>Raspberry Cheesecake</v>
       </c>
       <c r="E2" t="str">
-        <v>تشيزكيك بالتوت</v>
+        <v/>
       </c>
       <c r="F2" t="str">
-        <v>Frambuazli premium cheesecake</v>
+        <v>Taze frambuaz ile hazırlanmış kremsi cheesecake. 12 dilim.</v>
       </c>
       <c r="G2" t="str">
-        <v>Himbeer-Kasekuchen Premium</v>
+        <v>Cremiger Käsekuchen mit frischen Himbeeren. 12 Stück.</v>
       </c>
       <c r="H2" t="str">
-        <v>Raspberry premium cheesecake</v>
+        <v>Creamy cheesecake with fresh raspberries. 12 slices.</v>
       </c>
       <c r="I2" t="str">
-        <v>تشيزكيك فاخر بالتوت</v>
+        <v/>
       </c>
       <c r="J2" t="str">
         <v>Pastalar</v>
@@ -487,22 +528,37 @@
         <v>Cheesecake</v>
       </c>
       <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
         <v>Donuk</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>kutu</v>
       </c>
-      <c r="N2">
+      <c r="O2">
         <v>18.5</v>
       </c>
-      <c r="O2">
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2">
         <v>12</v>
       </c>
-      <c r="P2">
+      <c r="S2">
         <v>8</v>
       </c>
-      <c r="Q2">
+      <c r="T2">
         <v>24</v>
+      </c>
+      <c r="U2">
+        <v>100</v>
+      </c>
+      <c r="V2">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -513,25 +569,25 @@
         <v>Mini Cookie Box</v>
       </c>
       <c r="C3" t="str">
-        <v>Mini Keksbox</v>
+        <v>Mini Cookie Box</v>
       </c>
       <c r="D3" t="str">
         <v>Mini Cookie Box</v>
       </c>
       <c r="E3" t="str">
-        <v>علبة كوكيز صغيرة</v>
+        <v/>
       </c>
       <c r="F3" t="str">
-        <v>Citir mini cookie kutusu</v>
+        <v/>
       </c>
       <c r="G3" t="str">
-        <v>Knusprige Mini-Keksbox</v>
+        <v/>
       </c>
       <c r="H3" t="str">
-        <v>Crispy mini cookie box</v>
+        <v/>
       </c>
       <c r="I3" t="str">
-        <v>علبة كوكيز صغيرة مقرمشة</v>
+        <v/>
       </c>
       <c r="J3" t="str">
         <v>Kurabiyeler</v>
@@ -540,27 +596,557 @@
         <v>Mini Kurabiyeler</v>
       </c>
       <c r="L3" t="str">
+        <v>Sweet Heaven</v>
+      </c>
+      <c r="M3" t="str">
         <v>Donuk olmayan</v>
       </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
         <v>koli</v>
       </c>
-      <c r="N3">
+      <c r="O3">
         <v>72</v>
       </c>
-      <c r="O3">
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3">
         <v>24</v>
       </c>
-      <c r="P3">
+      <c r="S3">
         <v>6</v>
       </c>
-      <c r="Q3">
+      <c r="T3">
         <v>30</v>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TIRAMISÙ-050</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Tiramisu Dilim</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Tiramisu Stück</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Tiramisu Slice</v>
+      </c>
+      <c r="E4" t="str">
+        <v>تيراميسو شريحة</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Gerçek mascarpone ile yapılmış klasik tiramisu. Bireysel porsiyonlar.</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Klassisches Tiramisu mit echtem Mascarpone. Einzelportionen.</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Classic tiramisu made with real mascarpone. Individual portions.</v>
+      </c>
+      <c r="I4" t="str">
+        <v>تيراميسو كلاسيكي مصنوع من الماسكاربوني الحقيقي.</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Pastalar</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Dilim Pastalar</v>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v>Donuk</v>
+      </c>
+      <c r="N4" t="str">
+        <v>adet</v>
+      </c>
+      <c r="O4">
+        <v>2.8</v>
+      </c>
+      <c r="P4">
+        <v>6.5</v>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4">
+        <v>10</v>
+      </c>
+      <c r="S4">
+        <v>10</v>
+      </c>
+      <c r="T4">
+        <v>20</v>
+      </c>
+      <c r="U4">
+        <v>50</v>
+      </c>
+      <c r="V4">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B41"/>
+  <cols>
+    <col min="1" max="1" width="38.83203125" customWidth="1"/>
+    <col min="2" max="2" width="90.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>başlık</v>
+      </c>
+      <c r="B1" t="str">
+        <v>açıklama</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>════  GENEL KURALLAR  ════</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Eşleştirme anahtarı</v>
+      </c>
+      <c r="B3" t="str">
+        <v>stok_kodu veritabanındaki mevcut ürünü bulur. Eşleşme olursa güncelleme yapılır; bulunamazsa yeni ürün oluşturulur.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Boş hücre = koru</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Boş bırakılan her hücre ESKİ DEĞERİ KORUR. O alan üzerinde hiçbir değişiklik yapılmaz.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Silmek için __CLEAR__</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Bir alanı sıfırlamak/silmek istiyorsanız hücreye tam olarak  __CLEAR__  yazın.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Bağımsız dil sütunları</v>
+      </c>
+      <c r="B6" t="str">
+        <v>tr / de / en / ar sütunları birbirinden bağımsızdır. Sadece güncellemek istediğiniz dili doldurun; diğerleri bozulmaz.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Sayısal format</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Fiyat ve adet sütunlarında nokta (.) ondalık ayracı olarak kullanın. Binlik ayraç (. veya ,) otomatik temizlenir.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v/>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>════  SÜTUN AÇIKLAMALARI  ════</v>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>stok_kodu</v>
+      </c>
+      <c r="B10" t="str">
+        <v>ZORUNLU. Ürünü veritabanında bulan benzersiz stok kodu. Hiçbir zaman değiştirmeyin.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>urun_adi_tr / de / en / ar</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Ürün adı (4 dil). Boş bırakılan dil mevcut adını korur. Yeni ürün oluşturulurken en az bir dil dolu olmalı.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>aciklama_tr / de / en / ar</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Ürün açıklaması (4 dil). Boş = korur. İstersen sadece Türkçe doldurup diğerlerini bırakabilirsin.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>kategori</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Ana kategori adı (bkz. "kategori_listesi" sayfası). Sistem yakın eşleşme yapar. Mevcut ürün güncelleniyorsa boş bırakabilirsin.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>alt_kategori</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Alt kategori adı. Yeni ürünün doğru konuma yerleşmesi için kullanılır. Boş = ana kategoriye düşer.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>tedarikci</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Tedarikçi şirket adı. Boş bırakılırsa içe aktarma panelinde seçilen tedarikçi kullanılır.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>urun_tipi</v>
+      </c>
+      <c r="B16" t="str">
+        <v>"Donuk"  veya  "Donuk olmayan". Nakliye ve gümrük hesaplamalarını etkiler. Boş = panelde seçilen tip kullanılır.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>alis_fiyat_seviyesi</v>
+      </c>
+      <c r="B17" t="str">
+        <v>"adet" | "kutu" | "koli" | "palet". Alış fiyatının hangi birime ait olduğunu belirtir. Bkz. aşağıdaki örnekler.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>alis_fiyati</v>
+      </c>
+      <c r="B18" t="str">
+        <v>EUR cinsinden alış fiyatı. Sistem bu değeri kutu başına normalize ederek satış fiyatlarını hesaplar. Boş = korur.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>satis_fiyati_musteri</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Müşteri satış fiyatı EUR (kutu başına). Dolu ise otomatik hesaplamayı DEVREDIŞİ bırakır. Boş = mevcut fiyat korunur.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>satis_fiyati_alt_bayi</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Alt bayi satış fiyatı EUR (kutu başına). Dolu ise otomatik hesaplamayı devre dışı bırakır. Boş = korur.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>kutu_ici_adet</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Bir kutudaki adet / dilim / porsiyon sayısı. Fiyat hesaplamalarının temel birimi.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>koli_ici_kutu</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Bir kolide kaç kutu olduğu. Koli bazlı fiyat çevirisinde kullanılır.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>palet_ici_koli</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Bir paletteki koli sayısı. Palet bazlı fiyat çevirisi için.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>stok_miktari</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Mevcut stok adedi (tam sayı). Boş = korur.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>aktif</v>
+      </c>
+      <c r="B25" t="str">
+        <v>1 = aktif (katalogda görünür)   |   0 = pasif (gizli). Boş = korur.</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v/>
+      </c>
+      <c r="B26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>════  ALIŞ FİYATI SEVİYESİ ÖRNEKLERİ  ════</v>
+      </c>
+      <c r="B27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>alis_fiyat_seviyesi: adet</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Örnek: kutu_ici_adet=12, alis_fiyati=1.50 → Kutu fiyatı = 1.50 × 12 = 18.00 EUR</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>alis_fiyat_seviyesi: kutu</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Örnek: alis_fiyati=18.50 → Kutu fiyatı direkt 18.50 EUR (en yaygın format)</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>alis_fiyat_seviyesi: koli</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Örnek: koli_ici_kutu=8, alis_fiyati=148.00 → Kutu fiyatı = 148.00 ÷ 8 = 18.50 EUR</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>alis_fiyat_seviyesi: palet</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Örnek: koli_ici_kutu=8, palet_ici_koli=24, alis_fiyati=3552 → Kutu = 3552 ÷ (8×24) = 18.50 EUR</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v/>
+      </c>
+      <c r="B32" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>════  KATEGORİ EŞLEŞTİRME  ════</v>
+      </c>
+      <c r="B33" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Nasıl çalışır?</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Sistem girilen kategori adını veritabanındaki slug ve isimlerle karşılaştırır. Tam eşleşme önceliklidir; bulunamazsa yakın eşleşme denenir.</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Örnek eşleşmeler</v>
+      </c>
+      <c r="B35" t="str">
+        <v>"pasta" → "Pastalar" ✓  |  "cheesecake" → "Cheesecake" ✓  |  "kuru pasta" → "Kurabiyeler" ✓</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Uyarı</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Yanlış eşleşme olursa ürün yanlış kategoriye düşer. Mevcut ürünleri güncellerken kategori sütununu boş bırakmak daha güvenlidir.</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Kategori listesi</v>
+      </c>
+      <c r="B37" t="str">
+        <v>"kategori_listesi" sayfasına bakın (elle doldurun veya veritabanından kopyalayın).</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v/>
+      </c>
+      <c r="B38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>════  TEKNİK ÖZELLİKLER  ════</v>
+      </c>
+      <c r="B39" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>gramaj, kalori vb.</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Ürüne özgü teknik özellikler (gramaj, kalori, allerjenler vb.) Excel üzerinden aktarılmaz; ürün detay sayfasından elle girilir.</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Paketleme verileri</v>
+      </c>
+      <c r="B41" t="str">
+        <v>kutu_ici_adet / koli_ici_kutu / palet_ici_koli sütunları teknik özellik tablosuna da yazılır; ayrıca girmenize gerek yok.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B41"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C8"/>
+  <cols>
+    <col min="1" max="1" width="55.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ana_kategori</v>
+      </c>
+      <c r="B1" t="str">
+        <v>alt_kategori</v>
+      </c>
+      <c r="C1" t="str">
+        <v>slug_ipucu</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Pastalar</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v>pastalar</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Pastalar</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Cheesecake</v>
+      </c>
+      <c r="C3" t="str">
+        <v>cheesecake</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Pastalar</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Dilim Pastalar</v>
+      </c>
+      <c r="C4" t="str">
+        <v>dilim-pastalar</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Kurabiyeler</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v>kurabiyeler</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Kurabiyeler</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Mini Kurabiyeler</v>
+      </c>
+      <c r="C6" t="str">
+        <v>mini-kurabiyeler</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>↑ Bu sayfa yalnızca referans içindir.</v>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Veritabanındaki gerçek kategori adlarını Admin › Ürün Yönetimi › Kategoriler sayfasından kopyalayın.</v>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>